<commit_message>
Strange New Worlds Final Episodes
</commit_message>
<xml_diff>
--- a/STARTREK.xlsx
+++ b/STARTREK.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4A104E-7468-4BA8-BC9D-A9949368A8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44313958-D358-4924-8AA0-979F7091E37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10671" uniqueCount="3822">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10673" uniqueCount="3824">
   <si>
     <t>id</t>
   </si>
@@ -11489,6 +11489,12 @@
   </si>
   <si>
     <t>2179.3</t>
+  </si>
+  <si>
+    <t>2355.6</t>
+  </si>
+  <si>
+    <t>2873.2</t>
   </si>
 </sst>
 </file>
@@ -19952,8 +19958,17 @@
       <c r="F168" t="s">
         <v>682</v>
       </c>
+      <c r="G168">
+        <v>49</v>
+      </c>
       <c r="H168" s="1">
         <v>46282</v>
+      </c>
+      <c r="I168" s="4" t="s">
+        <v>3822</v>
+      </c>
+      <c r="J168">
+        <v>2262</v>
       </c>
       <c r="K168" t="s">
         <v>21</v>
@@ -19993,8 +20008,17 @@
       <c r="F169" t="s">
         <v>685</v>
       </c>
+      <c r="G169">
+        <v>62</v>
+      </c>
       <c r="H169" s="1">
         <v>46289</v>
+      </c>
+      <c r="I169" s="4" t="s">
+        <v>3823</v>
+      </c>
+      <c r="J169">
+        <v>2262</v>
       </c>
       <c r="K169" t="s">
         <v>21</v>

</xml_diff>